<commit_message>
Export and style updated test summary report to Excel (.xlsx)
</commit_message>
<xml_diff>
--- a/multi-turn-context-manager/reports/tests/test_summary_06_22.xlsx
+++ b/multi-turn-context-manager/reports/tests/test_summary_06_22.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -482,6 +482,7 @@
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="45" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -532,10 +533,15 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Dịch Actual Result</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Technical Validation (Tiếng Việt)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Functional Evaluation (Tiếng Việt)</t>
         </is>
@@ -631,10 +637,46 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
+          <t>T1: Thời gian gọi: 105 giây.
+T2: Xin lỗi, nhưng chúng tôi không thể xác nhận thông tin đó từ tài liệu được cung cấp. Thông tin về người tham gia cuộc gọi GT_04 không được đề cập trong ngữ cảnh.
+T3: Id: f1f952e5-3369-4738-8e6d-4878a31af9d6, Session Id: GT_03, Ngày: 2026-05-03, Người tham gia: Shimada, Nakahara, Người nói: None, Thời gian gọi: 204 giây, Văn bản thô: A : Xin lỗi vì đã giữ anh chờ. Vâng, người phụ trách hiện tại không có mặt, vì vậy tôi muốn liên hệ lại với anh sau. Khi gọi lại, số điện thoại di động anh đang dùng có ổn không?  B : Vâng. À, hôm nay có gọi lại được không?
+A: À, tôi sẽ kiểm tra lại, nhưng có thể hôm nay sẽ khó. Vậy thì ngày mai hoặc sau có ổn không?
+B: À, tôi không chắc ngày mai có thể đi ra ngoài hay không, vì tôi có một số việc cần làm. À, về vấn đề này, tôi thấy có một tờ rơi ở gần đó với thông tin về Asset Japan và số điện thoại này, và nó nói rằng đây là một tài sản có thể bán.
+A: À, xin lỗi, đúng vậy.
+B: Và nó nói rằng tôi có thể gọi điện thoải mái, không có vấn đề gì.
+A: À, điều đó là đúng. Vâng.
+B: Tôi hiểu rồi. À, tôi không biết phải làm gì. À, tôi hiểu rồi, không có vấn đề.
+A: À, nhưng hôm nay hoặc ngày mai, tôi có thể gọi lại cho anh dưới dạng gọi lại không?
+B: Vâng, không có vấn đề.
+A: Tôi hiểu rồi. Và tôi sẽ gọi điện cho anh qua số điện thoại di động của anh. Xin lỗi, tôi có thể hỏi tên anh được không?
+B: Tôi là Shimada.
+A: À, Kumada ạ.
+B: À, tôi là Shimada.
+A: À, Shimada ạ.
+B: Vâng.
+A: À, xin lỗi. Cảm ơn anh. À, về vấn đề này, anh có thấy tờ rơi không?
+B: À, không, tôi đang đứng trước tài sản này.
+A: À, vậy à.
+B: Trước đó, tôi có thấy thông tin về tài sản này, nhưng bây giờ tôi không thấy nữa.
+A: Vâng
+B: Và tôi không biết liệu nó đã được bán hay chưa, vì vậy tôi muốn xem nội thất và nghe một số thông tin.
+A: À, tôi hiểu rồi. Về việc xem nội thất và liệu nó đã được bán hay chưa, tôi sẽ ghi chú lại.
+B: Vâng, đúng vậy.
+A: Tôi hiểu rồi. Vậy thì tôi sẽ chuyển thông tin này cho người phụ trách, và nếu hôm nay có thể gọi lại, tôi sẽ gọi lại. Nếu không, thì sẽ là ngày mai hoặc sau.
+B: Tôi hiểu rồi, không có vấn đề.
+A: Vâng, xin lỗi, cảm ơn anh.
+B: Vâng, xin cảm ơn.
+A: Vâng, xin lỗi.
+B: Tạm biệt., Tóm tắt: Tóm tắt cho GT_03.
+T4: Thời gian gọi: 105 giây.</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
           <t>Khởi tạo chủ đề (SQL) -&gt; Giải quyết đại từ (Heuristics) -&gt; Chuyển đổi chủ đề -&gt; Quay lại chủ đề cũ qua lịch sử hội thoại.</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Xác nhận luồng hội thoại đa lượt cốt lõi: từ việc bắt đầu chủ đề; giải quyết đại từ "ai/câu chuyện đó" đến việc chuyển đổi và khôi phục ngữ cảnh cũ thành công.</t>
         </is>
@@ -688,10 +730,15 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
+          <t>T1: Trong cuộc gọi GT_04, người nhận cuộc gọi (người nghe) không nêu rõ tên của mình.  Mặt khác, người đàn ông gọi điện (bên phát) tự giới thiệu là "Yokohori từ ngân hàng Mitsubishi UFJ". Do đó, tên của người nhận cuộc gọi (bên nhận) không thể được xác nhận từ thông tin được cung cấp.</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
           <t>Nhận diện thực thể mơ hồ (Tier 2)</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>Hệ thống nhận diện được "Anh ấy" có thể chỉ 2 người khác nhau và buộc phải dùng LLM Router để phân tích sâu thay vì dùng luật Heuristic đơn giản.</t>
         </is>
@@ -745,10 +792,15 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng chúng tôi không thể xác nhận thông tin đó từ tài liệu được cung cấp. Do không có kết quả tìm kiếm cụ thể hoặc siêu dữ liệu liên quan đến "ca sĩ A của thông tin" trong ngữ cảnh, chúng tôi không thể đưa ra câu trả lời chi tiết.</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
           <t>Định tuyến Pipeline (SQL -&gt; WEB)</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Kiểm tra khả năng phát hiện sự thay đổi ý định đột ngột của người dùng từ việc hỏi dữ liệu nội bộ sang tìm kiếm thông tin trên mạng.</t>
         </is>
@@ -820,10 +872,33 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
+          <t>T1: Id: 61819a9a-20c8-4767-bbb7-589a265def5d, Session Id: GT_02, Ngày: 2026-05-02, Người tham gia: Nakaoka, Ishida Shiho, Shiho, Ishida, Người nói: None, Thời gian gọi: 80 giây, Văn bản thô: A: Vâng, cảm ơn. Đây là Asset Japan.
+B: Tôi được sự giúp đỡ của quý vị. Tôi là Nakaoka từ Valtes.
+A: Vâng, tôi được sự giúp đỡ của quý vị.
+B: Tôi được sự giúp đỡ của quý vị. Hôm nay, ông Ishida từ bộ PMG có mặt không?
+A: Ông Ishida từ bộ PMG… ạ, tên cuối là gì?
+B: Vâng, ông Shiho.
+A: À, vâng. À, xin lỗi. Vì ông ấy đang ở nhà, nên tôi sẽ gọi lại, vậy tôi có thể xin số điện thoại của quý vị không?
+B: À, vâng. Tôi sẽ nói. 050
+A: 050, vâng.
+B: 1782
+A: 1782, vâng.
+B: 1880
+A: 1880, đúng. Vâng. Ông Nakaoka từ Valtes, đúng không?
+B: Xin lỗi. À, công ty của tôi là Valtes, với "Va" là đầu, "l" tiếp theo, "te" và "s" cuối cùng.
+A: Valtes. À, vâng, tôi xin lỗi.
+B: Xin lỗi. Vâng, xin cảm ơn.
+A: Vâng, tôi sẽ gọi lại. Xin cảm ơn.
+B: Vâng, tôi xin phép. Tạm biệt.
+A: Tạm biệt., Tóm tắt: Tóm tắt cho GT_02.</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
           <t>Khởi tạo phiên mới</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>Đảm bảo hệ thống khởi tạo đúng ngữ cảnh cho một ID phiên hoàn toàn mới; không bị lẫn lộn với dữ liệu cũ.</t>
         </is>
@@ -877,10 +952,15 @@
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi. Quá trình tạo câu trả lời đã hết thời gian. Vui lòng đợi một lát và thử lại.</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
           <t>Cơ chế ngắt mạch &amp; Fallback</t>
         </is>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>Đảm bảo hệ thống không bị treo khi AI chính chậm phản hồi; tự động chuyển sang phương án dự phòng (Heuristics/Embedding) để luôn có phản hồi.</t>
         </is>
@@ -934,10 +1014,15 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi. Thời gian chờ đã hết trong khi tạo câu trả lời. Vui lòng đợi một lát và thử lại.</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
           <t>Xử lý lỗi định dạng JSON</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>Xác nhận khả năng tự phục hồi của hệ thống khi mô hình ngôn ngữ trả về kết quả không đúng cấu trúc JSON mong đợi.</t>
         </is>
@@ -991,10 +1076,15 @@
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
+          <t>T1: Không tìm thấy dữ liệu phù hợp.</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
           <t>Xử lý lỗi chính tả (Typo Tolerance)</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="L8" s="3" t="inlineStr">
         <is>
           <t>Hệ thống hiểu và xử lý đúng các lỗi phát âm/chính tả tiếng Nhật (ví dụ: 'tsuuwa' thay vì 'tsuwa') thông qua ánh xạ ngữ nghĩa.</t>
         </is>
@@ -1048,10 +1138,15 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
+          <t>T1: Không tìm thấy dữ liệu phù hợp.</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
           <t>Xử lý trộn ngôn ngữ (Code-mixing)</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t>AI giải mã chính xác các thuật ngữ hỗn hợp Anh-Nhật ("call", "end") để ánh xạ vào đúng các trường dữ liệu của cuộc gọi.</t>
         </is>
@@ -1118,10 +1213,28 @@
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
+          <t>T1: Cuộc gọi giữa GT_04 và GT_06 khác nhau như sau:
+1. **Mục đích và bối cảnh**
+- **GT_04**: Ông Yokohori của ngân hàng Mitsubishi UFJ muốn liên lạc với bà Nakahara Rinka (làm thêm giờ) của Asset Japan với mục đích truyền đạt thông điệp. Vì bà Nakahara không đi làm trong ngày, ông yêu cầu truyền đạt thông điệp thay thế.
+- **GT_06**: Ông Yamashita của AJ Technologies kiểm tra tình hình có mặt của "ông Kase" (có thể là người phụ trách cụ thể) với người nói chuyện 1 (Esta) của công ty xây dựng. Ông Kase đang vắng mặt, và ông Yamashita đồng ý sẽ liên lạc lại.
+2. **Sự khác biệt về kết quả**
+- **GT_04**: Việc truyền đạt thông điệp được chấp thuận, và thông tin liên lạc cụ thể (số điện thoại) cũng như giờ làm việc (thứ 2-6: 9h-21h, thứ 7, chủ nhật và ngày lễ: 9h-17h) được ghi rõ.
+- **GT_06**: Xác nhận ông Kase đang vắng mặt, và ông Yamashita đồng ý sẽ liên lạc lại, với lời hứa sẽ theo dõi trong tương lai.
+3. **Cấu trúc đối thoại**
+- **GT_04**: Người gọi (ngân hàng) yêu cầu người nhận (Asset Japan) thực hiện một yêu cầu cụ thể (truyền đạt thông điệp), và người nhận chấp thuận yêu cầu đó.
+- **GT_06**: Người gọi (AJ Technologies) yêu cầu người nhận (Esta của công ty xây dựng) xác nhận, và người nhận thông báo rằng "ông Kase đang vắng mặt", và đạt được sự đồng ý về việc theo dõi trong tương lai.
+4. **Mối quan hệ**
+- **GT_04**: Liên lạc công việc giữa ngân hàng và công ty bất động sản.
+- **GT_06**: Xác nhận cá nhân giữa các công ty (AJ Technologies và công ty xây dựng) để liên lạc với ông Kase.
+    **Kết luận**: Cả hai cuộc gọi đều có mục đích chung là "xác nhận người kia vắng mặt và điều chỉnh phản hồi trong tương lai", nhưng **nội dung cụ thể (truyền đạt thông điệp so với hứa hẹn theo dõi) và mối quan hệ (liên lạc công việc so với xác nhận cá nhân)** là khác nhau.</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
           <t>So sánh đa thực thể</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
         <is>
           <t>Hệ thống nhận diện yêu cầu so sánh giữa hai tài liệu và thực hiện truy xuất đầy đủ thay vì dùng bộ nhớ đệm đơn lẻ.</t>
         </is>
@@ -1181,10 +1294,15 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
+          <t>T1: ['web_1781689180', 'chủ đề mặc định_1781689195', 'chủ đề mới_08']</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
           <t>Giải phóng bộ nhớ LRU (Limit=3)</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t>Xác nhận cơ chế dọn dẹp bộ nhớ: khi có chủ đề thứ 4; chủ đề cũ nhất (GT_04) bị xóa để giữ cho bộ nhớ luôn gọn nhẹ (tối đa 3 slot).</t>
         </is>
@@ -1238,10 +1356,15 @@
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng chúng tôi không thể xác nhận thông tin đó từ tài liệu được cung cấp.</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
           <t>Làm mới dữ liệu theo TTL</t>
         </is>
       </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
         <is>
           <t>Đảm bảo thông tin tạm thời (như giá chứng khoán) được cập nhật mới từ web nếu dữ liệu trong bộ nhớ đệm đã quá hạn.</t>
         </is>
@@ -1295,10 +1418,15 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
+          <t>T1: Trong cuộc gọi GT_04, người nhận cuộc gọi (người nghe) không nêu rõ tên của mình.  Mặt khác, người đàn ông gọi điện (bên phát) tự giới thiệu là "Yokohori từ ngân hàng Mitsubishi UFJ". Do đó, tên của người nhận cuộc gọi (bên nhận) không thể được xác nhận từ thông tin được cung cấp.</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
           <t>Truy xuất nhanh qua Entity Index</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t>Xác nhận Tier 1 có thể trả lời ngay lập tức nếu đại từ đã được đăng ký rõ ràng trong chỉ mục thực thể của phiên.</t>
         </is>
@@ -1352,10 +1480,15 @@
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng từ tài liệu được cung cấp, chúng tôi không thể xác nhận thông tin cụ thể về "AJ Technologies cuộc gọi". Nội dung trong ngữ cảnh chỉ bao gồm hồ sơ yêu cầu tìm kiếm ('Tìm kiếm cuộc gọi AJ Technologies') và thông báo lỗi ở định dạng JSON. Về nội dung thực tế của cuộc gọi hoặc kết quả tìm kiếm, dữ liệu không đủ.</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
           <t>Phục hồi lỗi Embedding</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>Hệ thống vẫn hoạt động ổn định và chuyển sang Tier 2 để xử lý yêu cầu ngay cả khi dịch vụ vector hóa gặp sự cố.</t>
         </is>
@@ -1409,10 +1542,15 @@
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng chúng tôi không thể xác nhận thông tin đó từ tài liệu được cung cấp. Vui lòng cho chúng tôi biết câu hỏi hoặc yêu cầu của bạn.</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
           <t>Chuẩn hóa câu hỏi trống</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>Xử lý an toàn các trường hợp người dùng gửi tin nhắn không có nội dung thực tế.</t>
         </is>
@@ -1495,10 +1633,55 @@
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng thông tin này không thể được xác nhận từ tài liệu được cung cấp. Dựa trên thông tin trong ngữ cảnh, tôi sẽ tạo lại câu trả lời chính xác và không chứa thông tin sai lệch hoặc suy đoán. 
+---
+### **Chi tiết cuộc gọi GT_04 (tạo lại)**
+#### **Tham gia**
+- **Yokohori** (nam, thuộc Mitsubishi UFJ Bank)
+- **Người phụ nữ phụ trách** (thuộc và tên không được đề cập rõ ràng, nhưng phản hồi như người nhận cuộc gọi)
+- **Nakahara Rinka** (nữ, nhân viên part-time của Asset Japan, không phải người nhận cuộc gọi nhưng được đề cập như một liên lạc)
+#### **Thời gian cuộc gọi**
+- **Ngày 4 tháng 5 năm 2026**
+#### **Tóm tắt cuộc gọi**
+1. **Lời chào và giới thiệu**
+- Người phụ nữ phụ trách trả lời "Đây là Asset Japan".
+- Yokohori (Mitsubishi UFJ Bank) giải thích "Tôi đang được hỗ trợ. Tôi muốn liên hệ với Nakahara Rinka, vì vậy tôi đã gọi điện".
+2. **Tình hình làm việc của Nakahara Rinka**
+- Người phụ nữ phụ trách trả lời "Hôm nay cô ấy nghỉ. Chưa đến làm việc..."
+- Yokohori hỏi "Sau khi cô ấy đến làm việc, tôi có thể yêu cầu cô ấy gọi lại cho ngân hàng của chúng tôi được không?"
+3. **Đồng ý với yêu cầu truyền đạt**
+- Người phụ nữ phụ trách đồng ý "Vâng, tôi đã hiểu".
+- Yokohori bổ sung "Tôi đã gọi điện cho Nakahara nhiều lần và để lại tin nhắn trên máy trả lời tự động với tên ngân hàng và số điện thoại, vì vậy cô ấy đã biết số điện thoại".
+4. **Xác nhận giờ làm việc của ngân hàng**
+- Yokohori giải thích "Giờ làm việc... của quầy tiếp nhận, từ 9 giờ sáng đến 21 giờ vào ngày thường. Thứ bảy, chủ nhật và ngày lễ từ 9 giờ sáng đến 17 giờ".
+- Người phụ nữ phụ trách xác nhận "21 giờ, vâng", "17 giờ, vâng".
+5. **Kết thúc cuộc gọi**
+- Yokohori chào "Xin lỗi vì sự bất tiện. Cảm ơn".
+- Người phụ nữ phụ trách trả lời "Xin lỗi".
+#### **Vị trí của người gọi và người nhận**
+- **Người gọi**: **Yokohori** (thuộc Mitsubishi UFJ Bank, nam)
+- **Người nhận**: **Người phụ nữ phụ trách** (phụ trách tiếp nhận điện thoại của Asset Japan, thuộc và tên không được đề cập rõ ràng)
+#### **Các điểm đồng ý quan trọng**
+- Đồng ý truyền đạt cho Nakahara Rinka (nhân viên part-time của Asset Japan) về việc nhận cuộc gọi từ Mitsubishi UFJ Bank.
+- Nội dung truyền đạt: "Yokohori từ Mitsubishi UFJ Bank muốn liên hệ".
+- Người phụ nữ phụ trách xác nhận "Tôi đã hiểu. Tôi sẽ truyền đạt".
+#### **Bổ sung**
+- Nakahara Rinka không làm việc vào ngày đó (4 tháng 5 năm 2026), vì vậy điện thoại được truyền đạt thông qua người phụ nữ phụ trách.
+- Giờ làm việc của Mitsubishi UFJ Bank (9:00 ~ 21:00 vào ngày thường, 9:00 ~ 17:00 vào thứ bảy, chủ nhật và ngày lễ) đã được xác nhận.
+---
+### **Lưu ý**
+- **Thuộc Asset Japan**: Người phụ nữ phụ trách trả lời "Đây là Asset Japan", nhưng danh sách tham gia không đề cập rõ ràng về "Asset Japan", vì vậy thông tin này là suy đoán từ nội dung cuộc gọi và không phải là thông tin chắc chắn.
+- **Thuộc của Nakahara Rinka**: Danh sách tham gia có "Nakahara Rinka" (nữ), nhưng thuộc và vị trí (nhân viên part-time) là suy đoán từ nội dung cuộc gọi.
+Trên đây là thông tin chính xác dựa trên ngữ cảnh. 
+*(Lưu ý: Câu trả lời này không hoàn toàn phù hợp với tự kiểm tra, vì vậy độ tin cậy thấp hơn.)*</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
           <t>Kiểm soát ảo giác (Self-check)</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>Hệ thống tự phát hiện câu trả lời không khớp với dữ liệu gốc và cảnh báo "độ tin cậy thấp" thay vì đưa ra thông tin sai.</t>
         </is>
@@ -1555,10 +1738,16 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
+          <t>T1: [3646.404999999504, 8193.688699999257, 13119.435099999464]
+T2: Lỗi thời gian chờ đã được kích hoạt</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
           <t>Advisory Locking &amp; Xếp hàng tuần tự</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t>Đảm bảo tính nhất quán dữ liệu; ngăn chặn tình trạng Race Condition (xung đột dữ liệu) khi nhiều yêu cầu xử lý cùng lúc trên một phiên.</t>
         </is>
@@ -1628,10 +1817,21 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
+          <t>T1: Ông Yokohori của ngân hàng Mitsubishi UFJ đã để lại lời nhắn cho **Nakahara Rinka**.      **Lý do**：
+- Ông Yokohori đã nói trong cuộc gọi "Tôi muốn thông báo một việc cho Nakahara Rinka, vì vậy tôi đã gọi điện" và chỉ rõ "Nakahara Rinka" là người nhận lời nhắn.
+- Người phụ nữ (Nữ) nhận cuộc gọi đã trả lời "Vâng, tôi đã chấp nhận" và chấp nhận yêu cầu nhắn tin cho Nakahara Rinka.
+- Danh sách tham gia có nhiều tên "Nakahara Rinka", "Rinka", "Nakahara", nhưng trong nội dung cuộc gọi, họ sử dụng tên đầy đủ "Nakahara Rinka" và đây là người nhận lời nhắn rõ ràng.      Do đó, lời nhắn của ông Yokohori được xác nhận là để lại cho **Nakahara Rinka**.
+T2: Theo tài liệu cung cấp, vào ngày 4 tháng 5 năm 2026, Nakahara Rinka không có mặt tại văn phòng. Người phụ nữ (Nữ) nhận cuộc gọi đã nói "Hôm nay là ngày nghỉ, chưa đến làm việc...". Điều này xác nhận Nakahara Rinka không có mặt tại văn phòng vào ngày đó.
+T3: Session Id: GT_02, Ngày: 2026-05-02, Tham gia: Nakaoka, Ishida Shiho, Shiho, Ishida, Tóm tắt: Tóm tắt cho GT_02.
+T4: Trong cuộc gọi của GT_04, tên của người đại diện ngân hàng Mitsubishi UFJ là **Yokohori**.    (Trong ngữ cảnh, người đàn ông (Nam) đã tự giới thiệu "Tôi là Yokohori của ngân hàng Mitsubishi UFJ".)</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
           <t>Suy luận nhân vật -&gt; Theo dõi đại từ -&gt; Đổi ngữ cảnh -&gt; Truy xuất bộ nhớ ngắn hạn</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>Kiểm chứng khả năng suy luận phức tạp: xác định nhân vật (Nakahara Rinka); theo dõi giới tính đại từ (Cô ấy); và nhớ lại tên đại diện công ty đã nhắc từ 3 lượt trước (Yokobori).</t>
         </is>
@@ -1693,10 +1893,21 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
+          <t>T1: Trong cuộc gọi GT_03, ông Shimada đã bày tỏ mong muốn xác nhận xem có thể xem nhà được không và liệu nó đã được bán hay chưa. Ngoài ra, ông đã gọi điện cho số điện thoại của Asset Japan được dán trên bưu kiện của tài sản với lý do "nếu có thể xem nhà, tôi muốn được nói chuyện và nghe nhiều điều" và do đó, cuối cùng đã đồng ý với liên lạc lại từ người phụ trách.
+T2: Trong cuộc gọi GT_03, về tình hình hiện tại của tài sản mà ông Shimada đã xác nhận, các thông tin sau được ghi trong bối cảnh:
+1. **Vị trí của tài sản**: Ông Shimada đã nói "hiện tại tôi đang đứng trước tài sản" và do đó, có thể xác nhận rằng tài sản vẫn còn tồn tại.
+2. **Thay đổi thông tin**: Ông Shimada đã nói "trước đây, có rất nhiều thông tin về bất động sản này được đăng tải, nhưng bây giờ không thể xem được nữa" và do đó, thông tin trực tuyến về tài sản đã được đăng tải trước đây nhưng hiện tại không được hiển thị.
+3. **Tình hình bán**: Ông Shimada đã nói "tôi không biết chắc chắn liệu nó đã được bán hay chưa, vì vậy, nếu có thể xem nhà, tôi muốn..." và do đó, không rõ liệu tài sản đã được bán hay chưa. 
+**Kết luận**: 
+Tài sản mà ông Shimada đã xác nhận vẫn còn tồn tại, và về việc liệu có thể xem nhà hay tình hình bán, người phụ trách (A) đã nói "sẽ ghi lại để kiểm tra xem có thể xem nhà được không, hoặc đã bán hay chưa" và ông Shimada đã đồng ý. Do đó, tình hình hiện tại chi tiết của tài sản (đã bán hay có thể xem nhà) sẽ phải chờ liên lạc lại từ người phụ trách, và từ bối cảnh không thể có được kết luận rõ ràng.</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
           <t>Theo dõi trạng thái thực thể (Bất động sản)</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="L19" s="3" t="inlineStr">
         <is>
           <t>Xác nhận khả năng đào sâu thông tin trong tài liệu RAG và duy trì theo dõi trạng thái của một đối tượng cụ thể qua nhiều lượt hỏi.</t>
         </is>
@@ -1753,10 +1964,19 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
+          <t>T1: Công ty tham gia chung trong các cuộc gọi GT_06, GT_07, GT_08 là **AJ Technologies**.
+- Trong **GT_06**, Yamashita của AJ Technologies là người gọi (bên gọi điện).
+- Trong **GT_07**, Yamashita của AJ Technologies là người nhận (bên nhận điện).
+- Trong **GT_08**, Tsuji của AJ Technologies là người nhận. 
+  Qua 3 cuộc gọi này, có thể xác nhận AJ Technologies tham gia.</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
           <t>Công cụ RAG lấy mẫu công bằng (Fair-Sampling)</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t>Xác nhận khả năng tổng hợp và so sánh thông tin chính xác từ 3 tài liệu khác nhau (AJ Technologies) cùng một lúc.</t>
         </is>
@@ -1814,10 +2034,16 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
+          <t>T1: Thời gian gọi: 660 giây.
+T2: Thời gian gọi: 660 giây.</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
           <t>Tổng hợp dữ liệu SQL (SUM/SORT)</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="L21" s="3" t="inlineStr">
         <is>
           <t>Đảm bảo AI có thể thực hiện các phép toán chính xác trên dữ liệu số (thời gian gọi) và sắp xếp kết quả thay vì chỉ đọc hiểu văn bản đơn thuần.</t>
         </is>
@@ -1877,10 +2103,17 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
+          <t>T1: Từ tài liệu được cung cấp, có thể xác nhận rằng Nakahara Rinka (なかはら りんか) đang làm việc bán thời gian tại công ty của quý vị (có thể là ngân hàng hoặc công ty liên quan). Ngoài ra, có ghi lại việc gọi điện nhiều lần và để lại thông điệp trên máy trả lời tự động với tên ngân hàng và số điện thoại. Tuy nhiên, không có thông tin chi tiết về bộ phận hoặc chức vụ của cô ấy, cũng như tình hình công việc hiện tại.  
+T2: Xin lỗi, nhưng không thể xác nhận thông tin về Shimada từ tài liệu được cung cấp.
+T3: Không, chúng khác nhau.   **Yokohori của GT_04** đã gọi điện để liên hệ với Nakahara Rinka của AJ Technologies từ ngân hàng Mitsubishi UFJ với mục đích liên lạc về hợp đồng hoặc công việc.    **Shimada của GT_03** đã gọi điện để kiểm tra tình hình bán hàng và xem nhà với mục đích liên quan đến bất động sản.      Mục đích của hai cuộc gọi là khác nhau (liên lạc ngân hàng vs kiểm tra bất động sản) và không giống nhau.</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
           <t>Quản lý bộ nhớ thực thể &amp; So sánh</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>AI thất bại do quá thận trọng khi không tìm thấy văn bản khẳng định trực tiếp về sự "khác biệt"; cho thấy ưu tiên tính an toàn tối đa.</t>
         </is>
@@ -1934,10 +2167,15 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng từ tài liệu được cung cấp, chúng tôi không thể xác nhận được tên của người nhận cuộc gọi GT_04. Trong nhật ký cuộc gọi, "Nữ (nữ giới)" là người phụ trách của Asset Japan đã trả lời, và cô ấy nói rằng cô ấy đã cố gắng gọi "Nakahara Rinka" là người nhận cuộc gọi, nhưng ngoài tên của "Nam (nam giới)" là Yokohori, tên của người nhận cuộc gọi không được đề cập.</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
           <t>Nhận diện thực thể mơ hồ (Tier 2)</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="L23" s="3" t="inlineStr">
         <is>
           <t>Hệ thống nhận diện được "Anh ấy" có thể chỉ 2 người khác nhau và buộc phải dùng LLM Router để phân tích sâu.</t>
         </is>
@@ -1991,10 +2229,15 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
+          <t>T1: Lỗi thời gian chờ đã được kích hoạt</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
           <t>An toàn phiên làm việc</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>Xác nhận hệ thống trả về lỗi TimeoutError đúng cách khi một yêu cầu bị giữ khóa quá lâu; tránh việc treo hệ thống vô hạn.</t>
         </is>
@@ -2056,10 +2299,15 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
+          <t>T1: Nhiều câu trả lời</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
           <t>Xử lý đồng thời đa nhiệm phức tạp</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="L25" s="3" t="inlineStr">
         <is>
           <t>Chứng minh hệ thống vẫn duy trì được độ chính xác và không nhầm lẫn dữ liệu khi xử lý song song 5 truy vấn đòi hỏi quét toàn bộ cơ sở dữ liệu.</t>
         </is>
@@ -2147,10 +2395,34 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng từ tài liệu được cung cấp, không thể xác nhận được thông tin về "mục đích cụ thể (để làm gì)" mà Yokohori-san đã liên hệ với Asset Japan trong cuộc gọi GT_04. Trong bối cảnh chỉ có ghi chú mơ hồ "điều muốn được hướng dẫn" và không có nội dung chi tiết nào được ghi lại.
+T2: Trong cuộc gọi GT_04, Nakahara Rinka (なかはら りんか) không có mặt tại công ty vào ngày đó. Người phụ nữ phụ trách (Nữ) đã nói trong cuộc gọi: "Hôm nay là ngày nghỉ. Chưa đến công ty, vì vậy ...". Điều này đã xác nhận Nakahara Rinka không có mặt tại công ty vào ngày đó (ngày nghỉ). Ngoài ra, người gọi (Nam) đã nói rằng Nakahara Rinka được biết đến là nhân viên part-time, và rõ ràng Nakahara Rinka là người nhận cuộc gọi (bên nhận điện thoại). Do đó, Nakahara Rinka không có mặt tại công ty vào ngày đó.
+T3: Session Id: GT_02, Ngày: 2026-05-02, Người tham gia: Nakaoka, Ishida Shiho, Shiho, Ishida, Tóm tắt: Tóm tắt cho GT_02.
+T4: Yokohori của GT_04 đã gọi điện từ **Ngân hàng Mitsubishi UFJ**. Điều này được xác nhận vì trong nhật ký cuộc gọi, anh ta đã tự giới thiệu mình là "Yokobori từ Ngân hàng Mitsubishi UFJ". Mặt khác, Nakaoka của GT_02 đã gọi điện từ công ty **Baltess**. Trong nhật ký cuộc gọi, anh ta giải thích rằng tên công ty bắt đầu bằng "Ba" của "Babibubebo", tiếp theo là "Ra" của "Lariru", sau đó là "Ta" của "Tachitsu", và cuối cùng là "Sa" của "Sashisu", và tên công ty này được xác định là "Baltess".
+T5: Khi đứng trước tài sản, hai điều mà Shimada-san quan tâm là:
+1. **Thông tin về tài sản đã được đăng tải trước đó nhưng hiện không thể xem được**
+- Shimada-san nói: "Trước đây, thông tin về tài sản này đã được đăng trên trang web, nhưng bây giờ không thể xem được nữa". Điều này cho thấy Shimada-san cảm thấy疑惑 về việc thông tin tài sản đột nhiên biến mất.
+2. **Trạng thái của tài sản, liệu nó đã được bán hay vẫn đang được bán, là không rõ ràng**
+- "Tôi không biết liệu nó đã được bán hay chưa, vì vậy tôi muốn xem nội thất và nghe các cuộc trò chuyện, v.v.", Shimada-san nói. Điều này cho thấy trạng thái của tài sản (đã bán hoặc đang bán) là không rõ ràng, và Shimada-san muốn xem nội thất và nghe giải thích chi tiết. 
+Hai điểm này là mối quan tâm chính của Shimada-san.
+T6: Shimada-san của GT_03 đã nói về các điểm sau:
+1. **Xác minh tài sản**: Xác minh số điện thoại của "Asset Japan" trên bưu kiện của tài sản và chỉ ra rằng nó có ghi "Xin vui lòng gọi điện thoải mái".
+2. **Điều chỉnh lịch**: Do có lịch trình khám bệnh vào ngày mai, có thể không thể trả lời điện thoại, vì vậy việc gọi lại sẽ được chuyển sang "ngày mai trở đi".
+3. **Mong muốn xem nội thất**: Ở trước tài sản, Shimada-san muốn xác minh tình trạng bán hàng và khả năng xem nội thất.
+4. **Cung cấp tên**: Shimada-san đã tiết lộ tên của mình là "Shimada" và tiến hành theo dòng chảy của cuộc gọi. 
+Cuối cùng, Shimada-san đã đồng ý với việc nhận cuộc gọi lại từ người phụ trách.
+T7: Asset Japan đã xuất hiện với vai trò **gọi điện (bên gọi điện)** trong cả hai cuộc gọi **GT_03** và **GT_09**.
+- Trong **GT_03**, người phụ trách của Asset Japan (A) đã gọi điện cho người được hỏi về việc xem nội thất và tình trạng bán hàng (B) và yêu cầu gọi lại.
+- Trong **GT_09**, ông Ito của Asset Japan (B) đã gọi điện cho người phụ trách của Bộ phận Quản lý Thanh toán Trung ương (A) và yêu cầu chuyển thông điệp về việc hỏi về tài sản ở Đông浦町 qua email. 
+Trong cả hai cuộc gọi, Asset Japan đều ở vị trí **gọi điện cho các công ty hoặc cá nhân khác với mục đích thực hiện các nghiệp vụ của mình (giới thiệu và hỏi về tài sản)**.</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
           <t>Phân giải đại từ đa lượt dài (7 lượt) + suy luận giới tính (彼女) + so sánh chéo đa session</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="L26" s="3" t="inlineStr">
         <is>
           <t>Phân giải đại từ đa lượt dài (7 lượt) + suy luận giới tính (彼女) + so sánh chéo đa session</t>
         </is>
@@ -2224,10 +2496,23 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
+          <t>T1: Thời gian gọi: 250 giây.
+T2: Id phiên: GT_03, thời gian gọi: 204 giây.
+T3: Dưới đây là Id phiên của các cuộc gọi ngắn dưới 60 giây:    **GT_05, GT_06, GT_07, GT_08, GT_09**      Thông tin này dựa trên kết quả thực hiện truy vấn SQL được đề cập trong ngữ cảnh.
+T4: Xin lỗi, nhưng không thể xác nhận thông tin đó từ tài liệu được cung cấp.    Tên và đơn vị của người tham gia trong cả hai cuộc trò chuyện GT_03 và GT_09 không được chỉ định rõ ràng.    Trong GT_03, tên "Shimada" và "Kumada" (sau đó được sửa thành "Shimada") xuất hiện, và trong GT_09, "Ito" xuất hiện, nhưng những người này là khác nhau và không có người nào tham gia cả hai cuộc trò chuyện.
+T5: Dưới đây là Id phiên của các cuộc gọi được thực hiện từ ngày 1 tháng 5 năm 2026 đến ngày 4 tháng 5:
+- **GT_01**
+- **GT_02**
+- **GT_03**
+- **GT_04**      Thông tin này được lấy từ kết quả thực hiện truy vấn SQL trong ngữ cảnh được cung cấp.</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
           <t>Truy vấn SQL phức tạp (SUM, MAX, COUNT, INTERSECT, BETWEEN)</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="L27" s="3" t="inlineStr">
         <is>
           <t>Truy vấn SQL phức tạp (SUM, MAX, COUNT, INTERSECT, BETWEEN)</t>
         </is>
@@ -2313,10 +2598,31 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng thông tin đó không được xác nhận từ tài liệu được cung cấp.    （Lưu ý：Người dùng đã nhập `'; DROP TABLE transcripts; --` là mã giả SQL Injection và không liên quan đến ngữ cảnh này.）      ---    **Nội dung cuộc gọi GT_03（trích）**
+- **Thời gian**: Ngày 3 tháng 5 năm 2026
+- **Tham gia**:
+- Shimada（nam）
+- Nakahara（nam, thuộc AJ Technologies）
+T2: Xin lỗi, nhưng thông tin về giá bán chính xác của tài sản đó không được xác nhận từ tài liệu được cung cấp. Nội dung cuộc trò chuyện không bao gồm mô tả về giá.
+T3: Xin lỗi, nhưng từ tài liệu được cung cấp, không rõ ràng về nội dung hoặc bối cảnh cụ thể mà "vấn đề đó" ám chỉ. Có nhiều cuộc trò chuyện trong ngữ cảnh, nhưng không có thông tin cụ thể để xác định chủ đề hoặc sự kiện được đề cập. Bạn có thể cung cấp câu hỏi hoặc thông tin bổ sung cụ thể hơn không？
+T4: Tóm tắt: Tóm tắt cho GT_09。
+T5: Shimada muốn các điểm sau：
+1. **Xác nhận tình trạng tài sản**：
+- 「Không rõ liệu nó đã được bán hay chưa」（muốn xác nhận xem tài sản vẫn còn được bán hay đã được bán）
+- 「Nếu có thể xem bên trong, tôi muốn nghe các cuộc trò chuyện và các thông tin khác」（muốn xem bên trong tài sản và nghe giải thích chi tiết về việc bán）
+2. **Muốn liên lạc**：
+- 「Liệu hôm nay hoặc ngày mai, có thể liên lạc lại được không？」（muốn người phụ trách liên lạc lại, nhưng nói rằng có thể hôm nay hoặc ngày mai）
+3. **Con đường thu thập thông tin**：
+- 「Gần đây, tôi đã xem thông tin về bất động sản đó, nhưng bây giờ không thể xem được nữa」（trước đây đã xem thông tin về tài sản trên trang web bất động sản, nhưng bây giờ không thể xem được, vì vậy muốn xác nhận trực tiếp）      Tóm lại, Shimada
+T6: Xin lỗi, nhưng thông tin đó không được xác nhận từ tài liệu được cung cấp.</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
           <t>Phòng vệ tấn công (SQL Injection, Data Mutation), kiểm soát ảo giác (Hallucination), trộn ngôn ngữ, lọc ký tự vô nghĩa</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="L28" s="3" t="inlineStr">
         <is>
           <t>Phòng vệ tấn công (SQL Injection, Data Mutation), kiểm soát ảo giác (Hallucination), trộn ngôn ngữ, lọc ký tự vô nghĩa</t>
         </is>
@@ -2381,10 +2687,17 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
+          <t>T1: Ông Yamashita đã gọi điện với lý do không được mô tả trực tiếp trong tài liệu cung cấp. Tuy nhiên, trong nhật ký cuộc gọi GT_06, có phát biểu "Ông Kase có trở về không?" từ đó có thể suy đoán ông Yamashita gọi điện để xác nhận sự vắng mặt của ông Kase. Ngoài ra, trong cuộc gọi GT_07, có vẻ như ông Yamashita gọi điện với mục đích đề xuất một kế hoạch mới, nhưng đây là một cuộc trò chuyện khác (GT_07). Do đó, mục đích của cuộc gọi điện của ông Yamashita trong GT_06 có thể được coi là "xác nhận sự vắng mặt của ông Kase", nhưng đây là suy đoán từ ngữ cảnh và không có mô tả rõ ràng.
+T2: Trong GT_07, nội dung chính mà ông Yamashita (thuộc AJ Technologies) muốn truyền đạt cho người nhận cuộc gọi (Marcken) là "đề xuất một kế hoạch mới". Cụ thể, ông Yamashita nói "Tôi muốn mang lại một kế hoạch mới" và cuộc trò chuyện tiếp tục với việc xác nhận nội dung. Tuy nhiên, vì Marcken trả lời "Không có ở đây", ông Yamashita nói "Tôi sẽ gọi lại qua điện thoại di động" và kết thúc cuộc gọi. **Vị trí của người gọi và người nhận** - **Người gọi (người gọi điện)**: Ông Yamashita (AJ Technologies) - **Người nhận (người nhận điện)**: Marcken (không rõ tên công ty hoặc thuộc) **Kết luận** Ông Yamashita gọi điện với mục đích đề xuất một kế hoạch mới và vì người nhận không có mặt, ông nói sẽ gọi lại.
+T3: Kết quả của cuộc gọi điện của ông Yamashita trong GT_06 và GT_07 như sau: **Kết quả của GT_06** Ông Yamashita (người gọi) đã xác nhận với người nhận (người nhận điện) về việc "Ông Kase" có trở về không, nhưng người nhận trả lời "Đang ra ngoài". Ông Yamashita nói "Tôi sẽ gọi lại" và kết thúc cuộc gọi. Trong cuộc gọi này, không có kết quả cụ thể (ví dụ: thỏa thuận hoặc quyết định hành động). **Kết quả của GT_07** Ông Yamashita (người gọi) đã xác nhận với người nhận (người nhận điện) về việc "Ông Ishihara" có trở về không và gọi điện với mục đích đề xuất một kế hoạch mới. Người nhận trả lời "Muốn họp vào thứ Tư, ngày 14, lúc 10 giờ" và ông Yamashita xác nhận "Đồng ý với thời gian đó". Trong cuộc gọi này, **đã thống nhất sẽ tổ chức họp vào thứ Tư, ngày 14, lúc 10 giờ**. Trên đây là kết quả của hai cuộc gọi điện của ông Yamashita.</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
           <t>Xử lý thực thể trùng tên (Disambiguation), so sánh đa ngữ cảnh</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="L29" s="3" t="inlineStr">
         <is>
           <t>Xử lý thực thể trùng tên (Disambiguation), so sánh đa ngữ cảnh</t>
         </is>
@@ -2467,10 +2780,38 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
+          <t>T1: Trong cuộc gọi GT_04, Yokohori (thuộc ngân hàng Mitsubishi UFJ) đã truyền đạt thông tin cụ thể như sau:
+1. **Mục đích liên lạc**
+- Yokohori của ngân hàng Mitsubishi UFJ đã gọi điện để thông báo cho Nakahara Rinka (hoặc "Rinka") đang làm việc tại Asset Japan về một vấn đề.
+2. **Lịch sử liên lạc trước đó**
+- Yokohori đã giải thích rằng đã gọi điện nhiều lần cho điện thoại di động của Nakahara Rinka và đã để lại lời nhắn trên máy trả lời tự động với "tên ngân hàng và số điện thoại".
+3. **Giờ làm việc**
+- Yokohori đã thông báo về giờ làm việc của ngân hàng Mitsubishi UFJ như sau:
+- **Thứ hai đến thứ sáu**: 9 giờ sáng đến 9 giờ tối
+- **Thứ bảy, chủ nhật và ngày lễ**: 9 giờ sáng đến 5 giờ chiều
+4. **Nội dung yêu cầu truyền đạt**
+- Yokohori đã yêu cầu người trả lời điện thoại (người nghe cuộc gọi) truyền đạt cho Nakahara Rinka rằng "muốn gọi điện sau khi đi làm".
+- "Nếu có thể, tôi có thể yêu cầu người khác truyền đạt, vậy có thể yêu cầu gọi điện cho tôi không?"
+5. **Yêu cầu cuối cùng**
+- "Rất xin lỗi vì sự bất tiện, nhưng xin cảm ơn". 
+    --- 
+    **Bổ sung**
+- Yokohori (người gọi) đang yêu cầu người trả lời điện thoại (người nghe cuộc gọi) truyền đạt thông tin cho Nakahara Rinka (người nhận) với mục đích liên lạc trực tiếp.
+- Nội dung truyền đạt bao gồm cả giờ làm việc của ngân hàng và xác nhận liên lạc, với giả định rằng Nakahara Rinka sẽ "nhận điện thoại sau khi đi làm". 
+| T2: Trong cuộc gọi GT_04, giờ làm việc được ghi lại như sau:
+- **Thứ hai đến thứ sáu**: 9 giờ sáng đến 9 giờ tối
+- **Thứ bảy, chủ nhật và ngày lễ**: 9 giờ sáng đến 5 giờ chiều 
+    Thông tin này được Yokohori (người gọi) của ngân hàng Mitsubishi UFJ truyền đạt để thông báo cho Nakahara Rinka (người nhận). 
+| T3: Xin lỗi, nhưng không thể xác nhận thông tin về mã nhân viên (hoặc số nhận dạng tương tự) của Yokohori từ tài liệu được cung cấp. Không có ghi chú tương ứng trong ngữ cảnh. 
+| T4: Ito của GT_09 thuộc công ty **Asset Japan** tại thành phố Nagoya, tỉnh Aichi. Thông tin này được xác nhận từ lời tự giới thiệu của B (Ito) trong nhật ký cuộc gọi.</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
           <t>Tái sử dụng bộ đệm (Cache reuse), self-check phát hiện thông tin thiếu, tự động phục hồi khi embedding lỗi</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="L30" s="3" t="inlineStr">
         <is>
           <t>Tái sử dụng bộ đệm (Cache reuse), self-check phát hiện thông tin thiếu, tự động phục hồi khi embedding lỗi</t>
         </is>
@@ -2524,10 +2865,15 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
+          <t>T1: 5 câu trả lời đã nhận được</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
           <t>Tranh chấp Advisory Lock, xếp hàng tuần tự</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="L31" s="3" t="inlineStr">
         <is>
           <t>Tranh chấp Advisory Lock, xếp hàng tuần tự</t>
         </is>
@@ -2593,10 +2939,20 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
+          <t>T1: Xin lỗi, nhưng từ tài liệu được cung cấp, chúng tôi không thể xác nhận được nội dung cụ thể hoặc bản ghi cuộc gọi của "GT_99". Dữ liệu cuộc trò chuyện trong bối cảnh chỉ giới hạn ở các phiên "GT_01", "GT_02", "GT_03" và không tìm thấy thông tin liên quan đến GT_99.
+T2: Xin lỗi, nhưng từ tài liệu được cung cấp, chúng tôi không thể xác nhận thông tin đó. Bối cảnh không chứa số liệu cụ thể hoặc thông tin mới nhất về "giá cổ phiếu của ngân hàng Mitsubishi UFJ hôm nay". Ngoài ra, còn có lỗi định dạng JSON, điều này có thể dẫn đến thất bại trong việc thu thập dữ liệu. Để có thông tin chính xác hơn, có thể cần phải tìm kiếm lại từ nguồn khác hoặc tại thời điểm khác.
+T3: Xin lỗi, nhưng từ tài liệu được cung cấp, chúng tôi không thể xác nhận được giải thích hoặc nội dung liên quan đến "trọng thuyết". Trong bối cảnh, từ "giải thích" chỉ xuất hiện một lần, nhưng từ "trọng thuyết" không xuất hiện và cũng không tìm thấy bất kỳ ghi chú nào về định nghĩa hoặc nội dung của nó.
+T4: a=Xin lỗi, tôi đã cung cấp thông tin sai. Thông tin chính xác dựa trên bối cảnh như sau:
+b=Xin lỗi, nhưng từ tài liệu được cung cấp, chúng tôi không thể xác nhận thông tin đó. Về cách làm mì ramen ngon,
+c= Những người tham gia cuộc họp GT_05 bao gồm **Sakamoto** (nam) và **Kumagai** (nam), tổng cộng 2 người.</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
           <t>Xử lý session không tồn tại, tự động chuyển đổi sang Web, phục hồi cache sau câu hỏi ngoài lề</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="L32" s="3" t="inlineStr">
         <is>
           <t>Xử lý session không tồn tại, tự động chuyển đổi sang Web, phục hồi cache sau câu hỏi ngoài lề</t>
         </is>

</xml_diff>